<commit_message>
Actualiza dashboard: mejoras Campanas/Mapa, README y flujo
</commit_message>
<xml_diff>
--- a/Data/Bitacora.xlsx
+++ b/Data/Bitacora.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.100.136\reporteria\Documentación CDG\4 CARLOS\ARCHIVO ALERTAS\Scotiabank_Proyeccion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fastcogroupchile-my.sharepoint.com/personal/clorcat_fastcogroup_com/Documents/Escritorio/Scotiabank/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40BF20F4-3B0A-42B7-A546-CEDEE9A721AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{40BF20F4-3B0A-42B7-A546-CEDEE9A721AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B61BA39-3552-4233-B25C-5FD006775130}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{8BD92864-C893-40BB-ABD1-D31D2B15F0A2}"/>
   </bookViews>
@@ -93,12 +93,21 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="12">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_ &quot;$&quot;* #,##0_ ;_ &quot;$&quot;* \-#,##0_ ;_ &quot;$&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="167" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="168" formatCode="_ &quot;$&quot;* #,##0.00_ ;_ &quot;$&quot;* \-#,##0.00_ ;_ &quot;$&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="169" formatCode="_ \$* #,##0_ ;_ \$* \-#,##0_ ;_ \$* \-_ ;_ @_ "/>
+    <numFmt numFmtId="170" formatCode="_ &quot;$&quot;* #,##0_ ;_ &quot;$&quot;* \-#,##0_ ;_ &quot;$&quot;* \-_ ;_ @_ "/>
+    <numFmt numFmtId="171" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
+    <numFmt numFmtId="172" formatCode="_-* #,##0_-;\-* #,##0_-;_-* \-_-;_-@_-"/>
+    <numFmt numFmtId="173" formatCode="0\ %"/>
+    <numFmt numFmtId="174" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * \-_ ;_ @_ "/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -127,8 +136,170 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Aptos Display"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -153,8 +324,181 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -162,12 +506,548 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="429">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="170" fontId="17" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="17" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="171" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="172" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
+    <xf numFmtId="173" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="173" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="173" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
+    <xf numFmtId="173" fontId="21" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -198,10 +1078,438 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="43" fontId="0" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="429">
+    <cellStyle name="20% - Énfasis1" xfId="18" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis1 2" xfId="85" xr:uid="{9A54C635-D808-4B86-B8A5-AEBBE6F237A5}"/>
+    <cellStyle name="20% - Énfasis1 3" xfId="301" xr:uid="{5808F3BB-70C9-48E9-B619-AE6FA9023155}"/>
+    <cellStyle name="20% - Énfasis2" xfId="21" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis2 2" xfId="87" xr:uid="{4B7DD14E-8DF8-437A-A811-F76D76A03172}"/>
+    <cellStyle name="20% - Énfasis2 3" xfId="303" xr:uid="{D8A30880-684E-423B-BB31-DDF022DC2C97}"/>
+    <cellStyle name="20% - Énfasis3" xfId="24" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis3 2" xfId="89" xr:uid="{0540579B-7764-42CE-B4C4-2CB61AE5F334}"/>
+    <cellStyle name="20% - Énfasis3 3" xfId="305" xr:uid="{2DA81152-D361-4FB4-B9C0-5CF127C6F3EA}"/>
+    <cellStyle name="20% - Énfasis4" xfId="27" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis4 2" xfId="91" xr:uid="{20FF4BE5-4F12-4676-B626-794EA7ECDC0A}"/>
+    <cellStyle name="20% - Énfasis4 3" xfId="307" xr:uid="{802D6791-12F2-456B-BC3E-E5509252A2C3}"/>
+    <cellStyle name="20% - Énfasis5" xfId="30" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis5 2" xfId="93" xr:uid="{5A3CC8FA-0169-4E4E-A93A-6BF27F32BD0B}"/>
+    <cellStyle name="20% - Énfasis5 3" xfId="309" xr:uid="{CC2BFE84-5FE8-419C-9F15-431F9104684E}"/>
+    <cellStyle name="20% - Énfasis6" xfId="33" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis6 2" xfId="95" xr:uid="{33BDAC27-9674-4626-B73E-C78E0D582FCE}"/>
+    <cellStyle name="20% - Énfasis6 3" xfId="311" xr:uid="{6E37DE20-D542-4999-83E8-0FB8E9A8CBB4}"/>
+    <cellStyle name="40% - Énfasis1" xfId="19" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis1 2" xfId="86" xr:uid="{B03BD32F-337C-4476-B43F-E209D9AD1588}"/>
+    <cellStyle name="40% - Énfasis1 3" xfId="302" xr:uid="{D65A2B8E-CE7A-4832-83AB-E31D88BBF465}"/>
+    <cellStyle name="40% - Énfasis2" xfId="22" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis2 2" xfId="88" xr:uid="{3B666CC2-3815-4853-8399-0988CE37FBB3}"/>
+    <cellStyle name="40% - Énfasis2 3" xfId="304" xr:uid="{F24104E4-B28B-45C3-932F-378DFD36C397}"/>
+    <cellStyle name="40% - Énfasis3" xfId="25" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis3 2" xfId="90" xr:uid="{4012B3DA-4962-4DE1-8F86-B2B9EC69C6C7}"/>
+    <cellStyle name="40% - Énfasis3 3" xfId="306" xr:uid="{EAFD6B11-DA38-49F0-9492-B33683A05EC6}"/>
+    <cellStyle name="40% - Énfasis4" xfId="28" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis4 2" xfId="92" xr:uid="{04DD6EAA-BA69-41F9-883A-2A399CF3C55D}"/>
+    <cellStyle name="40% - Énfasis4 3" xfId="308" xr:uid="{E24B141E-637D-4222-B8BB-59C75C96D96E}"/>
+    <cellStyle name="40% - Énfasis5" xfId="31" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis5 2" xfId="94" xr:uid="{A9E5B6EC-C8CD-4F84-BE4B-D2DD2C795D05}"/>
+    <cellStyle name="40% - Énfasis5 3" xfId="310" xr:uid="{CC078BE9-3B47-490C-92AA-3F976EC545DB}"/>
+    <cellStyle name="40% - Énfasis6" xfId="34" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis6 2" xfId="96" xr:uid="{04C730AD-9A44-4A0C-82DF-5B5869178664}"/>
+    <cellStyle name="40% - Énfasis6 3" xfId="312" xr:uid="{0B256993-E472-455F-86F8-D51ED9046B1B}"/>
+    <cellStyle name="60% - Énfasis1 2" xfId="39" xr:uid="{26DAC7C7-6CB5-4B8D-906A-1F0EA8BB432C}"/>
+    <cellStyle name="60% - Énfasis2 2" xfId="40" xr:uid="{70541E63-166C-4071-A34F-0EF2E86EC88C}"/>
+    <cellStyle name="60% - Énfasis3 2" xfId="41" xr:uid="{AF96D0A2-C4F6-4618-8AD6-0B34C95932C4}"/>
+    <cellStyle name="60% - Énfasis4 2" xfId="42" xr:uid="{3C807D4B-C673-483D-BA3A-707C47A7E632}"/>
+    <cellStyle name="60% - Énfasis5 2" xfId="43" xr:uid="{85E3A36D-54A9-422B-AA6E-69B329599CB6}"/>
+    <cellStyle name="60% - Énfasis6 2" xfId="44" xr:uid="{D9B53077-B3DD-4FFE-B0D0-F5DAE5E1D5CD}"/>
+    <cellStyle name="Bueno" xfId="7" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Encabezado 1" xfId="3" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Encabezado 4" xfId="6" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Énfasis1" xfId="17" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Énfasis2" xfId="20" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Énfasis3" xfId="23" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Énfasis4" xfId="26" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Énfasis5" xfId="29" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Énfasis6" xfId="32" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Excel Built-in Comma [0]" xfId="248" xr:uid="{DDED3304-B1CB-4020-9C6B-6FFBBE88831A}"/>
+    <cellStyle name="Excel Built-in Currency [0]" xfId="71" xr:uid="{724873F8-3188-439A-8DB6-F1891E42D8D7}"/>
+    <cellStyle name="Excel Built-in Currency [0] 1" xfId="70" xr:uid="{71479855-ED13-49A7-BC4F-94B193AB15BC}"/>
+    <cellStyle name="Excel Built-in Currency [0] 1 2" xfId="141" xr:uid="{0D3A9F47-E6C3-441E-B5A4-A0C992769DDC}"/>
+    <cellStyle name="Excel Built-in Currency [0] 2" xfId="193" xr:uid="{43B65F24-9A32-4676-8F9B-011CCB80AE5F}"/>
+    <cellStyle name="Excel Built-in Currency [0] 3" xfId="226" xr:uid="{47EA50D9-C827-4DE2-94D5-5DA8CF67F552}"/>
+    <cellStyle name="Excel Built-in Currency [0] 4" xfId="208" xr:uid="{2E288E23-3C36-48E5-8720-793539BF4563}"/>
+    <cellStyle name="Hipervínculo 2" xfId="214" xr:uid="{6A8522F8-A6DA-43C5-956F-875868E6196A}"/>
+    <cellStyle name="Incorrecto" xfId="8" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
+    <cellStyle name="Millares [0] 10" xfId="240" xr:uid="{E784B494-140A-42BE-A8B7-BDDC1962477A}"/>
+    <cellStyle name="Millares [0] 10 2" xfId="350" xr:uid="{9F8DF67D-8EE5-4247-9313-19850345780E}"/>
+    <cellStyle name="Millares [0] 10 3" xfId="340" xr:uid="{C5DB8848-F188-4371-8C74-6B85CA02A095}"/>
+    <cellStyle name="Millares [0] 11" xfId="351" xr:uid="{1FFB38EA-2CAA-446B-9F0F-698BD57298E5}"/>
+    <cellStyle name="Millares [0] 2" xfId="216" xr:uid="{5A4F1191-E47F-4D4F-984E-B23B382F89DA}"/>
+    <cellStyle name="Millares [0] 3" xfId="212" xr:uid="{0AB021CD-D6FD-4AB3-A91B-B515AF85D6E8}"/>
+    <cellStyle name="Millares [0] 3 2" xfId="243" xr:uid="{B96C41BF-5A1F-407D-A633-600D53E45A3A}"/>
+    <cellStyle name="Millares [0] 3 2 2" xfId="353" xr:uid="{092431D8-807F-43AB-995C-015DEB6D3742}"/>
+    <cellStyle name="Millares [0] 3 2 3" xfId="343" xr:uid="{04AD2A3B-5CE6-4247-BCEF-FC67BAADF6F4}"/>
+    <cellStyle name="Millares [0] 3 3" xfId="245" xr:uid="{C32C97D6-1B26-434B-A796-674AD3E36A87}"/>
+    <cellStyle name="Millares [0] 3 3 2" xfId="354" xr:uid="{5741218A-4BC5-4E69-AD85-E9D4AB0DB90C}"/>
+    <cellStyle name="Millares [0] 3 3 3" xfId="345" xr:uid="{B4D244C2-A0E2-468D-B465-A4F406CC06E0}"/>
+    <cellStyle name="Millares [0] 3 4" xfId="352" xr:uid="{FBD6454B-B312-47D2-9DD5-68AD5BA24490}"/>
+    <cellStyle name="Millares [0] 3 5" xfId="326" xr:uid="{A7F4C849-A39B-4E79-B7B0-40F82E5CF5F9}"/>
+    <cellStyle name="Millares [0] 4" xfId="228" xr:uid="{5A29ACDC-28C7-4748-9CA8-50CCD1975586}"/>
+    <cellStyle name="Millares [0] 4 2" xfId="246" xr:uid="{F8BE97F5-A97F-418C-B51C-E08285DB3768}"/>
+    <cellStyle name="Millares [0] 4 2 2" xfId="356" xr:uid="{208DD395-AD45-475E-B34B-8FB2D27BF762}"/>
+    <cellStyle name="Millares [0] 4 2 3" xfId="346" xr:uid="{D4B72E48-1799-4F85-8D98-8E28A45BDA18}"/>
+    <cellStyle name="Millares [0] 4 3" xfId="355" xr:uid="{4E456652-FF2F-4B55-9BE5-600939738206}"/>
+    <cellStyle name="Millares [0] 4 4" xfId="328" xr:uid="{972404A7-C392-4C5E-8D4B-ADB625893E20}"/>
+    <cellStyle name="Millares [0] 5" xfId="230" xr:uid="{F47EC90D-F341-443A-96CB-B08408E43B63}"/>
+    <cellStyle name="Millares [0] 5 2" xfId="357" xr:uid="{6DA4C1FF-75BF-458B-9003-AED42FFE6B05}"/>
+    <cellStyle name="Millares [0] 5 3" xfId="330" xr:uid="{6F48358E-7162-43F1-9F44-DEE12716FE80}"/>
+    <cellStyle name="Millares [0] 6" xfId="232" xr:uid="{43F6385D-4A09-464F-8B2E-B5299F82A5ED}"/>
+    <cellStyle name="Millares [0] 6 2" xfId="358" xr:uid="{C3B20ADB-3CE7-4BB7-992E-13EDBFE4B504}"/>
+    <cellStyle name="Millares [0] 6 3" xfId="332" xr:uid="{B41D23E6-75BE-4C28-AD11-5B22EF1FDBD4}"/>
+    <cellStyle name="Millares [0] 7" xfId="234" xr:uid="{C1F7C63C-CD92-4DFB-899F-18E55053FB73}"/>
+    <cellStyle name="Millares [0] 7 2" xfId="359" xr:uid="{8F5C3E4B-1B7C-42FD-920E-84D1AC5BBCCF}"/>
+    <cellStyle name="Millares [0] 7 3" xfId="334" xr:uid="{99B73419-E6FA-4BCD-9CBF-ABB6A50FDA48}"/>
+    <cellStyle name="Millares [0] 8" xfId="236" xr:uid="{394C810B-3EEC-425A-965F-98D7BD7DB197}"/>
+    <cellStyle name="Millares [0] 8 2" xfId="360" xr:uid="{708299E9-CFCF-4219-81B9-BED2A48B794C}"/>
+    <cellStyle name="Millares [0] 8 3" xfId="336" xr:uid="{073B5B8A-F276-4283-9EE2-CEEBFFD0262E}"/>
+    <cellStyle name="Millares [0] 9" xfId="238" xr:uid="{2347052E-3455-4724-8C80-5AD6D2BAA603}"/>
+    <cellStyle name="Millares [0] 9 2" xfId="361" xr:uid="{38884FF3-B7F9-40AB-A2A2-841708A6B415}"/>
+    <cellStyle name="Millares [0] 9 3" xfId="338" xr:uid="{61DD40A1-490D-4CBE-BB32-8833E6059D82}"/>
+    <cellStyle name="Millares 2" xfId="135" xr:uid="{93CC600F-572D-4928-811D-9750640403EA}"/>
+    <cellStyle name="Millares 2 2" xfId="215" xr:uid="{14A51E1F-7B4F-4C05-8C59-BE510D1DBC49}"/>
+    <cellStyle name="Moneda [0] 10" xfId="73" xr:uid="{74DB0B0E-8C72-4EC3-9990-6D1B20263F21}"/>
+    <cellStyle name="Moneda [0] 10 2" xfId="130" xr:uid="{54A71410-92B5-4ADB-8007-E321EE383FB9}"/>
+    <cellStyle name="Moneda [0] 10 2 2" xfId="362" xr:uid="{74BD7D1C-ED00-4E3A-B812-91366DC265E9}"/>
+    <cellStyle name="Moneda [0] 10 3" xfId="235" xr:uid="{01C6BF3E-392D-48AA-8D32-11426CF898F3}"/>
+    <cellStyle name="Moneda [0] 10 4" xfId="271" xr:uid="{8CB596C1-A636-4DE3-92F8-5ABC77C9A912}"/>
+    <cellStyle name="Moneda [0] 10 5" xfId="335" xr:uid="{AC35BCE4-A3A0-4593-9F53-A9A06CEA3359}"/>
+    <cellStyle name="Moneda [0] 11" xfId="75" xr:uid="{63DD16F2-F0F5-4B01-8CB3-1A1682856D86}"/>
+    <cellStyle name="Moneda [0] 11 10" xfId="237" xr:uid="{1CC76C08-15AD-4421-B4CA-3D2D5B58AF10}"/>
+    <cellStyle name="Moneda [0] 11 11" xfId="272" xr:uid="{1C11B07E-7AFD-4738-ADF7-6FAB65791845}"/>
+    <cellStyle name="Moneda [0] 11 12" xfId="337" xr:uid="{D0F192EC-775C-441A-AFE6-663BFB679E52}"/>
+    <cellStyle name="Moneda [0] 11 2" xfId="98" xr:uid="{172ECAB8-B097-4625-8E50-777F0F5D1CCA}"/>
+    <cellStyle name="Moneda [0] 11 2 2" xfId="278" xr:uid="{C3CCD564-3922-41CA-B993-B57D188A3376}"/>
+    <cellStyle name="Moneda [0] 11 2 3" xfId="363" xr:uid="{E3840816-8AF5-4614-A90A-D6DBD357FA67}"/>
+    <cellStyle name="Moneda [0] 11 3" xfId="100" xr:uid="{B17CC657-F071-4AA6-BEE5-CB99CC4BD842}"/>
+    <cellStyle name="Moneda [0] 11 3 2" xfId="279" xr:uid="{2B2853A8-97B0-4A51-895C-AC47D2CD61A6}"/>
+    <cellStyle name="Moneda [0] 11 4" xfId="102" xr:uid="{9A0AFCD2-7FA3-4080-9FBD-1097E4ABED88}"/>
+    <cellStyle name="Moneda [0] 11 4 2" xfId="280" xr:uid="{4A5AC7B1-09E8-49EA-9755-BFE0BF90D41F}"/>
+    <cellStyle name="Moneda [0] 11 5" xfId="104" xr:uid="{03351C36-4705-4BB5-AE31-EBB10576A7B1}"/>
+    <cellStyle name="Moneda [0] 11 5 2" xfId="281" xr:uid="{1FFDCB86-D37C-44E7-A5AB-2C5CE24677BF}"/>
+    <cellStyle name="Moneda [0] 11 6" xfId="106" xr:uid="{64F2CB75-40D8-4944-A994-3B4A8F29235C}"/>
+    <cellStyle name="Moneda [0] 11 6 2" xfId="282" xr:uid="{6C6A0A63-2E3D-4C16-948B-F5717408B88C}"/>
+    <cellStyle name="Moneda [0] 11 7" xfId="108" xr:uid="{79BBE230-5344-438A-9A86-2AB5924F2893}"/>
+    <cellStyle name="Moneda [0] 11 7 2" xfId="283" xr:uid="{C5DE552B-6F4A-4034-AEA5-C10E0496C389}"/>
+    <cellStyle name="Moneda [0] 11 8" xfId="110" xr:uid="{4508FB20-F7D2-408A-BABC-5D154A1043C8}"/>
+    <cellStyle name="Moneda [0] 11 8 2" xfId="284" xr:uid="{3D02F4C4-4A7A-4F9E-8596-3832E292FD3E}"/>
+    <cellStyle name="Moneda [0] 11 9" xfId="155" xr:uid="{D1B10050-9F64-40CA-B6D1-5020FE573204}"/>
+    <cellStyle name="Moneda [0] 12" xfId="77" xr:uid="{57CC0D46-36A1-4452-91E3-8B08D831F99B}"/>
+    <cellStyle name="Moneda [0] 12 2" xfId="156" xr:uid="{0029FC6B-4279-4E9B-8DFA-C97368C739DB}"/>
+    <cellStyle name="Moneda [0] 12 2 2" xfId="364" xr:uid="{9CA95061-FAE8-4FA4-9F63-11B1C95E58F1}"/>
+    <cellStyle name="Moneda [0] 12 3" xfId="239" xr:uid="{4A191A35-9708-4B2B-AE91-B181EA53BC13}"/>
+    <cellStyle name="Moneda [0] 12 4" xfId="273" xr:uid="{22B340E5-A97D-476C-8173-EF3AAC649FA0}"/>
+    <cellStyle name="Moneda [0] 12 5" xfId="339" xr:uid="{6E7BA6DF-06AE-48BB-B98D-DC46D4813FBD}"/>
+    <cellStyle name="Moneda [0] 13" xfId="79" xr:uid="{ECB9E8F3-639E-440B-B605-ABD531B4074D}"/>
+    <cellStyle name="Moneda [0] 13 2" xfId="157" xr:uid="{D617335A-35E5-4C2F-8C2A-304B30E84F29}"/>
+    <cellStyle name="Moneda [0] 13 2 2" xfId="365" xr:uid="{8A957F76-9FCE-4126-A090-2D2F325FF575}"/>
+    <cellStyle name="Moneda [0] 13 3" xfId="241" xr:uid="{6E9B79B3-5DE9-4A0F-AD39-352EB42B21D2}"/>
+    <cellStyle name="Moneda [0] 13 4" xfId="274" xr:uid="{734A75D1-62C8-4EC1-AE98-C6B8391FBEF8}"/>
+    <cellStyle name="Moneda [0] 13 5" xfId="341" xr:uid="{7437E553-A6BD-4059-9D90-AAE1EFE34603}"/>
+    <cellStyle name="Moneda [0] 14" xfId="81" xr:uid="{F3C7510E-95B5-4EA0-BA69-9C8ED5FAA154}"/>
+    <cellStyle name="Moneda [0] 14 2" xfId="158" xr:uid="{D883CEEE-757E-4644-98AD-47735E3D0BBC}"/>
+    <cellStyle name="Moneda [0] 14 3" xfId="217" xr:uid="{263F5CB5-69EA-48E5-A4C5-83D3F020EFC0}"/>
+    <cellStyle name="Moneda [0] 14 4" xfId="275" xr:uid="{260AADE5-9F6A-4270-9349-DD0ABFA4CF9B}"/>
+    <cellStyle name="Moneda [0] 15" xfId="112" xr:uid="{34CA95D9-3F52-47ED-9993-70551A578E2B}"/>
+    <cellStyle name="Moneda [0] 15 2" xfId="159" xr:uid="{276F963E-39E9-4945-8D23-B889FC283DAC}"/>
+    <cellStyle name="Moneda [0] 15 2 2" xfId="366" xr:uid="{C2AD4016-0570-498F-B1E7-C95DEF899A33}"/>
+    <cellStyle name="Moneda [0] 15 3" xfId="244" xr:uid="{8AEC9501-14F5-493A-A3FD-D89D15B27AE2}"/>
+    <cellStyle name="Moneda [0] 15 4" xfId="285" xr:uid="{871C647D-DDF9-48DA-A4DE-DC3B6C400AAA}"/>
+    <cellStyle name="Moneda [0] 15 5" xfId="344" xr:uid="{E06E371B-B498-4206-98DC-967DBCAB37CE}"/>
+    <cellStyle name="Moneda [0] 16" xfId="114" xr:uid="{729918CE-639A-4D08-87DB-4BCE55E69FBF}"/>
+    <cellStyle name="Moneda [0] 16 2" xfId="160" xr:uid="{C1AB8FAB-5671-423B-87B6-61E51A0775FA}"/>
+    <cellStyle name="Moneda [0] 16 2 2" xfId="367" xr:uid="{A877330C-C833-486D-96E0-49FF924DE77C}"/>
+    <cellStyle name="Moneda [0] 16 3" xfId="247" xr:uid="{823B02BD-977F-4122-A943-C39739166A50}"/>
+    <cellStyle name="Moneda [0] 16 4" xfId="286" xr:uid="{D2C1C29D-A4DD-48D1-8090-238BC2F2AB2F}"/>
+    <cellStyle name="Moneda [0] 16 5" xfId="347" xr:uid="{3810E475-8B73-47D2-BFA5-F50D72601727}"/>
+    <cellStyle name="Moneda [0] 17" xfId="116" xr:uid="{624125A0-0522-49CA-80B6-D040220EB603}"/>
+    <cellStyle name="Moneda [0] 17 2" xfId="161" xr:uid="{C801EEE6-94C3-4671-A987-BB9339076A40}"/>
+    <cellStyle name="Moneda [0] 17 2 2" xfId="378" xr:uid="{F9D3437B-715B-46AF-BB6C-2DACE5E4034F}"/>
+    <cellStyle name="Moneda [0] 17 3" xfId="249" xr:uid="{9615C858-1F32-4831-9E10-A81CC72896A9}"/>
+    <cellStyle name="Moneda [0] 17 3 2" xfId="380" xr:uid="{01628EEE-46CF-4E11-991E-F2FC5830094A}"/>
+    <cellStyle name="Moneda [0] 17 4" xfId="287" xr:uid="{84A042A3-EEA2-492F-BE12-AD57A14859FC}"/>
+    <cellStyle name="Moneda [0] 17 5" xfId="348" xr:uid="{F70DCD75-0A76-45D7-B791-1C46AB4E1039}"/>
+    <cellStyle name="Moneda [0] 18" xfId="118" xr:uid="{BB9CA380-058D-43C7-AEB5-CFD959FEB667}"/>
+    <cellStyle name="Moneda [0] 18 2" xfId="162" xr:uid="{AD442207-F0FD-4F18-962A-BCBAB380E9AA}"/>
+    <cellStyle name="Moneda [0] 18 3" xfId="288" xr:uid="{720DBAAD-0A37-4E3F-8D72-6DEA086BE372}"/>
+    <cellStyle name="Moneda [0] 18 4" xfId="349" xr:uid="{1F9DC7A4-6946-49F6-B7B9-9ADC9ECD993C}"/>
+    <cellStyle name="Moneda [0] 19" xfId="120" xr:uid="{5054C975-BDEF-4F2B-A90A-4481BF04A36C}"/>
+    <cellStyle name="Moneda [0] 19 2" xfId="289" xr:uid="{6172EA5D-63DD-4B1D-8A59-9B28223BFFD7}"/>
+    <cellStyle name="Moneda [0] 19 3" xfId="379" xr:uid="{2F4EA637-9402-47BF-ABD1-722B526ACB55}"/>
+    <cellStyle name="Moneda [0] 2" xfId="49" xr:uid="{5971C588-F3F4-462A-9B00-D8C59749A36E}"/>
+    <cellStyle name="Moneda [0] 2 10" xfId="187" xr:uid="{93B24E05-EE78-4731-9AB9-5EE680D5CBE3}"/>
+    <cellStyle name="Moneda [0] 2 11" xfId="131" xr:uid="{65EDA7B2-1E60-458A-A68D-39F9BC17A79A}"/>
+    <cellStyle name="Moneda [0] 2 12" xfId="209" xr:uid="{6A16DC5F-3C5B-4B43-AF34-4B51A600AE60}"/>
+    <cellStyle name="Moneda [0] 2 13" xfId="259" xr:uid="{76F61A4B-8E3A-4470-9CE1-C86FCD3DD2E0}"/>
+    <cellStyle name="Moneda [0] 2 14" xfId="323" xr:uid="{2A1AB2F8-6959-456A-9D76-373C152F5F24}"/>
+    <cellStyle name="Moneda [0] 2 2" xfId="65" xr:uid="{B3652B75-A82D-4848-81F8-025CB8916900}"/>
+    <cellStyle name="Moneda [0] 2 2 2" xfId="169" xr:uid="{037F3C0E-9A51-42DD-8BA7-DD33ED2FD1E8}"/>
+    <cellStyle name="Moneda [0] 2 2 3" xfId="174" xr:uid="{6360F5D7-E98B-4BB9-8BFF-22D1B7A9BE9A}"/>
+    <cellStyle name="Moneda [0] 2 2 4" xfId="180" xr:uid="{9CB86215-03AE-4323-AF91-1D57E4000B0F}"/>
+    <cellStyle name="Moneda [0] 2 2 5" xfId="190" xr:uid="{305FCBC7-C613-43F8-89A9-E1D7EA656D96}"/>
+    <cellStyle name="Moneda [0] 2 2 6" xfId="142" xr:uid="{760DF3D2-EF4E-47EB-83B8-9C3EC2A8E690}"/>
+    <cellStyle name="Moneda [0] 2 2 7" xfId="218" xr:uid="{49E1817E-E778-43C5-BEA9-DCEF5F5AEECF}"/>
+    <cellStyle name="Moneda [0] 2 2 8" xfId="270" xr:uid="{29C784BD-170C-4293-9826-E5C8FC368317}"/>
+    <cellStyle name="Moneda [0] 2 3" xfId="83" xr:uid="{8D17E258-F6A1-4AB9-B0AF-0B879B32AD61}"/>
+    <cellStyle name="Moneda [0] 2 3 2" xfId="192" xr:uid="{7C14D08F-1CB4-4F50-AB4F-1D1808A7801B}"/>
+    <cellStyle name="Moneda [0] 2 3 3" xfId="145" xr:uid="{6E6D7A98-6492-432A-B5E3-8758F8E1E834}"/>
+    <cellStyle name="Moneda [0] 2 3 4" xfId="277" xr:uid="{38145D7E-32C4-4FED-8251-E5C366D6EA89}"/>
+    <cellStyle name="Moneda [0] 2 3 5" xfId="368" xr:uid="{FBF2229D-80A6-4AE7-BBAB-4C592693C362}"/>
+    <cellStyle name="Moneda [0] 2 4" xfId="149" xr:uid="{94CFA73D-5224-4911-A3DD-CAC558712F9A}"/>
+    <cellStyle name="Moneda [0] 2 4 2" xfId="299" xr:uid="{2FD36573-FBBE-4DAD-87B1-1B75E3A6FA87}"/>
+    <cellStyle name="Moneda [0] 2 5" xfId="152" xr:uid="{764A2A1E-D96C-4511-9CB6-7492122DAC91}"/>
+    <cellStyle name="Moneda [0] 2 6" xfId="166" xr:uid="{D6162D4E-489B-465F-92D0-720231204E8C}"/>
+    <cellStyle name="Moneda [0] 2 7" xfId="172" xr:uid="{ED7E0D61-6298-4BE4-AE9E-1F707C2561EC}"/>
+    <cellStyle name="Moneda [0] 2 8" xfId="177" xr:uid="{B8E0A3CA-FB85-47EB-82DE-718A7324583D}"/>
+    <cellStyle name="Moneda [0] 2 9" xfId="183" xr:uid="{A5530265-CC78-4309-87B7-A4067F2D2843}"/>
+    <cellStyle name="Moneda [0] 20" xfId="122" xr:uid="{FAAE97C0-D9BA-41ED-914D-4535D2F0F672}"/>
+    <cellStyle name="Moneda [0] 20 2" xfId="290" xr:uid="{EA383C6C-4E33-4538-9798-2EA341746ACE}"/>
+    <cellStyle name="Moneda [0] 21" xfId="124" xr:uid="{7C742E4C-3E15-486F-A245-EA4EF947D760}"/>
+    <cellStyle name="Moneda [0] 21 2" xfId="291" xr:uid="{07EB3F32-37EE-48F9-BF0C-8D4F44C74607}"/>
+    <cellStyle name="Moneda [0] 22" xfId="46" xr:uid="{1B5FA973-E9F6-4132-80C2-DE45EC53CE99}"/>
+    <cellStyle name="Moneda [0] 22 2" xfId="293" xr:uid="{E5979B28-CEFA-41A7-B7C0-861949DE06B1}"/>
+    <cellStyle name="Moneda [0] 23" xfId="194" xr:uid="{1659CCFD-2705-4B16-B33C-4B14CD88DC2E}"/>
+    <cellStyle name="Moneda [0] 23 2" xfId="295" xr:uid="{BCB76D65-DA41-4F70-BA77-3F97694EFCDE}"/>
+    <cellStyle name="Moneda [0] 24" xfId="207" xr:uid="{4E200C61-5A45-412E-A99B-6690A8834F61}"/>
+    <cellStyle name="Moneda [0] 24 2" xfId="297" xr:uid="{C6B57AB8-0282-4FD1-8DB3-F9F7C43DC68C}"/>
+    <cellStyle name="Moneda [0] 25" xfId="314" xr:uid="{61612D46-9514-4D31-AA92-3271070EF8C0}"/>
+    <cellStyle name="Moneda [0] 26" xfId="316" xr:uid="{C77D6490-0967-4802-B605-1CF2B222C284}"/>
+    <cellStyle name="Moneda [0] 27" xfId="318" xr:uid="{FCDB31B3-4244-499A-A93F-715439D5BD58}"/>
+    <cellStyle name="Moneda [0] 28" xfId="320" xr:uid="{4E629AEF-96BE-450C-A40A-DDB4CC4499A9}"/>
+    <cellStyle name="Moneda [0] 29" xfId="322" xr:uid="{7D908D43-8DFD-473E-8961-A178E8FAC8C5}"/>
+    <cellStyle name="Moneda [0] 3" xfId="51" xr:uid="{09E37AFE-5497-4A22-848E-DECE4311CCFE}"/>
+    <cellStyle name="Moneda [0] 3 10" xfId="143" xr:uid="{96A08C07-9850-40E8-B280-E9005581FB62}"/>
+    <cellStyle name="Moneda [0] 3 11" xfId="210" xr:uid="{319C7BD7-5108-4229-9E16-F97520C88347}"/>
+    <cellStyle name="Moneda [0] 3 12" xfId="260" xr:uid="{7D6F6428-75C1-4C56-9779-89EC0AE90AB6}"/>
+    <cellStyle name="Moneda [0] 3 13" xfId="324" xr:uid="{79220DD3-B1A2-4D7B-B43B-06C712032331}"/>
+    <cellStyle name="Moneda [0] 3 2" xfId="64" xr:uid="{DB2FC025-A1D6-49FB-8E85-6725C98ACE02}"/>
+    <cellStyle name="Moneda [0] 3 2 2" xfId="146" xr:uid="{D0D81362-E790-4311-B49D-6EDFF326F86E}"/>
+    <cellStyle name="Moneda [0] 3 2 2 2" xfId="370" xr:uid="{B4C99731-11D5-46AB-819A-778D4E344416}"/>
+    <cellStyle name="Moneda [0] 3 2 3" xfId="242" xr:uid="{25779752-2500-4A6D-BB9E-B89DC5A2CDF6}"/>
+    <cellStyle name="Moneda [0] 3 2 4" xfId="269" xr:uid="{EB58183C-0A7D-44C9-B2CF-86D2EBD1DB87}"/>
+    <cellStyle name="Moneda [0] 3 2 5" xfId="342" xr:uid="{EF64E06C-94FA-4BAB-AB31-CC50B4DEAD5B}"/>
+    <cellStyle name="Moneda [0] 3 3" xfId="82" xr:uid="{12B592AB-1340-4EDE-B223-8E854174272A}"/>
+    <cellStyle name="Moneda [0] 3 3 2" xfId="150" xr:uid="{898D93CE-424A-48EE-9C5B-7086797B67F9}"/>
+    <cellStyle name="Moneda [0] 3 3 3" xfId="276" xr:uid="{C7E73288-EB08-462B-A500-7C2369830986}"/>
+    <cellStyle name="Moneda [0] 3 3 4" xfId="369" xr:uid="{53B32F05-DB2B-4EB8-A36C-74FC9F0BB3D6}"/>
+    <cellStyle name="Moneda [0] 3 4" xfId="153" xr:uid="{BAC44A2D-3FBE-426C-9F3E-94EADB0B772A}"/>
+    <cellStyle name="Moneda [0] 3 4 2" xfId="298" xr:uid="{A7932C82-80C0-4FDC-8755-CE317216F622}"/>
+    <cellStyle name="Moneda [0] 3 5" xfId="164" xr:uid="{7A4FE45C-A32B-468E-B09A-296024EB8FD9}"/>
+    <cellStyle name="Moneda [0] 3 5 2" xfId="184" xr:uid="{01406974-44CE-44F9-AA9D-B9484262960D}"/>
+    <cellStyle name="Moneda [0] 3 5 3" xfId="188" xr:uid="{21109479-1808-41EC-B02F-23CDE108C443}"/>
+    <cellStyle name="Moneda [0] 3 6" xfId="170" xr:uid="{08D5B548-F501-4080-A3A4-8E2CB96CD576}"/>
+    <cellStyle name="Moneda [0] 3 7" xfId="175" xr:uid="{07522EBE-CB91-4F75-8940-3E01579FC43A}"/>
+    <cellStyle name="Moneda [0] 3 8" xfId="181" xr:uid="{4A93AE8D-9879-4C7B-B536-3BDA62A78062}"/>
+    <cellStyle name="Moneda [0] 3 9" xfId="185" xr:uid="{81FFB747-FD91-42CA-BB97-285772DDAD0E}"/>
+    <cellStyle name="Moneda [0] 30" xfId="35" xr:uid="{27275856-C655-4F1E-A9B4-CBCF9B1CE11E}"/>
+    <cellStyle name="Moneda [0] 4" xfId="53" xr:uid="{8135222D-916D-421D-855E-76FA122DF69F}"/>
+    <cellStyle name="Moneda [0] 4 2" xfId="168" xr:uid="{1ACE625D-833F-450F-931D-D2730752FC71}"/>
+    <cellStyle name="Moneda [0] 4 2 2" xfId="371" xr:uid="{A9194220-5623-41D3-B22A-43FE33D1CE92}"/>
+    <cellStyle name="Moneda [0] 4 3" xfId="173" xr:uid="{7D1D126E-62C8-4153-A146-D922719C9F0C}"/>
+    <cellStyle name="Moneda [0] 4 4" xfId="179" xr:uid="{70414A1D-5585-4CF3-9AE1-172F5C22AE8C}"/>
+    <cellStyle name="Moneda [0] 4 5" xfId="189" xr:uid="{97A70A91-3AD8-4C51-A2A8-31E2FD58199C}"/>
+    <cellStyle name="Moneda [0] 4 6" xfId="133" xr:uid="{891C9868-31FD-4F17-9187-7A09B1AB9E69}"/>
+    <cellStyle name="Moneda [0] 4 7" xfId="211" xr:uid="{06AF58AD-5A3B-4078-8017-A22B0DFE9C4D}"/>
+    <cellStyle name="Moneda [0] 4 8" xfId="261" xr:uid="{E6784FED-CEB1-4D7B-B4F1-0AA3F6299E34}"/>
+    <cellStyle name="Moneda [0] 4 9" xfId="325" xr:uid="{11B297ED-20C9-4543-8A17-4330C450A1C8}"/>
+    <cellStyle name="Moneda [0] 5" xfId="55" xr:uid="{C1299496-9195-4B59-90D3-09605C351831}"/>
+    <cellStyle name="Moneda [0] 5 2" xfId="191" xr:uid="{08C52909-4687-4F98-BD39-192C4E5EA289}"/>
+    <cellStyle name="Moneda [0] 5 2 2" xfId="372" xr:uid="{615EBCB7-BCB4-408A-B3DE-A71B7ABA8C39}"/>
+    <cellStyle name="Moneda [0] 5 3" xfId="144" xr:uid="{D18D46A1-F766-4C06-AB36-CEB9C98F4A8A}"/>
+    <cellStyle name="Moneda [0] 5 4" xfId="227" xr:uid="{2EE56805-90FF-4B1D-9D8A-8952446B4CE0}"/>
+    <cellStyle name="Moneda [0] 5 5" xfId="262" xr:uid="{919139A8-148F-4804-9409-2E7BB3434072}"/>
+    <cellStyle name="Moneda [0] 5 6" xfId="327" xr:uid="{3ABFD6BF-674A-4CB4-8CE3-FE67C7C95046}"/>
+    <cellStyle name="Moneda [0] 6" xfId="57" xr:uid="{B6960A7F-C668-4743-A91C-3133B9882475}"/>
+    <cellStyle name="Moneda [0] 6 2" xfId="147" xr:uid="{F7F42303-3937-4446-AEE0-04B32D1687E9}"/>
+    <cellStyle name="Moneda [0] 6 2 2" xfId="220" xr:uid="{C4839A43-D686-445B-8CD3-FBB0B032DCEC}"/>
+    <cellStyle name="Moneda [0] 6 3" xfId="219" xr:uid="{56ED9C65-C8E5-4641-BEB2-1E0AFFD70066}"/>
+    <cellStyle name="Moneda [0] 6 4" xfId="264" xr:uid="{0D14CB6C-A615-405C-826A-A6305C6DD04E}"/>
+    <cellStyle name="Moneda [0] 7" xfId="59" xr:uid="{06BFB1EF-5D65-4514-B1DC-E6DD10FC893B}"/>
+    <cellStyle name="Moneda [0] 7 2" xfId="148" xr:uid="{BB20C4CE-E96B-4583-A643-ABDD08DFB3E1}"/>
+    <cellStyle name="Moneda [0] 7 2 2" xfId="373" xr:uid="{1996EDC2-5CEC-4D55-9B17-62F0D1B65B9E}"/>
+    <cellStyle name="Moneda [0] 7 3" xfId="229" xr:uid="{87762E9F-628B-492B-A48A-D850F90C772C}"/>
+    <cellStyle name="Moneda [0] 7 4" xfId="265" xr:uid="{D54E11DE-77E4-4A88-8264-0025B0CFD10F}"/>
+    <cellStyle name="Moneda [0] 7 5" xfId="329" xr:uid="{82105CB4-AAD5-4F93-982A-4D5C777114EC}"/>
+    <cellStyle name="Moneda [0] 8" xfId="61" xr:uid="{1B7E6E11-CE2D-4185-90E5-1C2B066BA606}"/>
+    <cellStyle name="Moneda [0] 8 2" xfId="151" xr:uid="{3F8398C3-6F6D-47E9-81BE-66DC24ED1A9C}"/>
+    <cellStyle name="Moneda [0] 8 2 2" xfId="374" xr:uid="{A6076530-3F7F-428E-9978-B628491D4531}"/>
+    <cellStyle name="Moneda [0] 8 3" xfId="231" xr:uid="{8766465F-653C-4A24-B057-CE280984645F}"/>
+    <cellStyle name="Moneda [0] 8 4" xfId="266" xr:uid="{85C3003D-7277-4523-A402-205A10EAD58C}"/>
+    <cellStyle name="Moneda [0] 8 5" xfId="331" xr:uid="{37C2A465-8001-4FA5-A872-41D7F024A92C}"/>
+    <cellStyle name="Moneda [0] 9" xfId="63" xr:uid="{1841603C-9064-4EF6-9922-22FA25BB42C8}"/>
+    <cellStyle name="Moneda [0] 9 2" xfId="154" xr:uid="{ED2B79AD-A4CA-4070-8AEE-B5F2B6F7BBC1}"/>
+    <cellStyle name="Moneda [0] 9 2 2" xfId="375" xr:uid="{A79DE2F2-70FD-4539-9E23-2B51D42F0A65}"/>
+    <cellStyle name="Moneda [0] 9 3" xfId="233" xr:uid="{F7AA24F3-A0CC-4121-9E5B-BB3C31DFDF06}"/>
+    <cellStyle name="Moneda [0] 9 4" xfId="268" xr:uid="{1535D1AD-2C7C-4F40-A38C-C566DABE511C}"/>
+    <cellStyle name="Moneda [0] 9 5" xfId="333" xr:uid="{D4D4093D-D57E-4911-ABB2-4651E3C4A08A}"/>
+    <cellStyle name="Moneda 10" xfId="197" xr:uid="{63E23AF0-5CE0-4A1D-99CF-6EC385AE02EA}"/>
+    <cellStyle name="Moneda 11" xfId="198" xr:uid="{1CD7DF67-CB5E-41CB-9339-A98274AE2431}"/>
+    <cellStyle name="Moneda 12" xfId="199" xr:uid="{830368D1-4352-4158-BEBE-1A9511A931E9}"/>
+    <cellStyle name="Moneda 13" xfId="200" xr:uid="{F9E60DAF-04E3-4A2C-8BCF-4390C2194429}"/>
+    <cellStyle name="Moneda 14" xfId="201" xr:uid="{EA92E611-F976-46CA-8735-5BC26A9183B0}"/>
+    <cellStyle name="Moneda 15" xfId="202" xr:uid="{6C3C2E82-E6B4-4092-A3D0-13DA3B48CF36}"/>
+    <cellStyle name="Moneda 16" xfId="203" xr:uid="{62317609-BB38-440F-B74B-9D89592C11A6}"/>
+    <cellStyle name="Moneda 17" xfId="204" xr:uid="{DE6C7B5B-AB81-4218-B6D5-10A7856185BA}"/>
+    <cellStyle name="Moneda 18" xfId="205" xr:uid="{0521C196-E98C-4CDB-A577-EA6C1CB72924}"/>
+    <cellStyle name="Moneda 19" xfId="206" xr:uid="{2D9348EC-7F82-4A4C-B98A-62CC4793A765}"/>
+    <cellStyle name="Moneda 2" xfId="36" xr:uid="{8D007098-4C2C-4DDE-BBC2-C8B1AAB6FCE0}"/>
+    <cellStyle name="Moneda 20" xfId="251" xr:uid="{4C530B17-022D-414E-8EFB-1BFF85694DBA}"/>
+    <cellStyle name="Moneda 21" xfId="252" xr:uid="{515751F0-C011-48E9-BBAE-0D14658AD7CA}"/>
+    <cellStyle name="Moneda 22" xfId="253" xr:uid="{E783A38C-4EDE-4853-8549-FBE8D13280B4}"/>
+    <cellStyle name="Moneda 23" xfId="254" xr:uid="{4DDDDE5B-CA18-48D6-9B0F-5034B21AC378}"/>
+    <cellStyle name="Moneda 24" xfId="255" xr:uid="{CD4732FB-23B7-4DC3-89CE-A4897A605DFC}"/>
+    <cellStyle name="Moneda 25" xfId="256" xr:uid="{DD4E039E-34F0-41AC-9820-C70D7A08E3A3}"/>
+    <cellStyle name="Moneda 26" xfId="267" xr:uid="{36DB358B-7221-4623-8FFF-22EB12E2BACB}"/>
+    <cellStyle name="Moneda 27" xfId="321" xr:uid="{BB0587EE-D173-4DA6-BD29-B5548738A3F7}"/>
+    <cellStyle name="Moneda 28" xfId="381" xr:uid="{5F0DF6E0-547A-40DA-BC52-213BE2B3E5C3}"/>
+    <cellStyle name="Moneda 29" xfId="382" xr:uid="{D39C44DC-4905-401B-94B5-ED588DE1D352}"/>
+    <cellStyle name="Moneda 3" xfId="37" xr:uid="{2528FFCF-E936-42E3-9507-BE9AF2278819}"/>
+    <cellStyle name="Moneda 30" xfId="383" xr:uid="{5F9FD1FF-4332-43A3-8DA4-EDA3DDA74110}"/>
+    <cellStyle name="Moneda 31" xfId="384" xr:uid="{29410D2C-5F67-438C-ADD9-FA10FDC8E9B1}"/>
+    <cellStyle name="Moneda 32" xfId="385" xr:uid="{ED1910B3-A602-448B-A8C6-0736A96F95E2}"/>
+    <cellStyle name="Moneda 33" xfId="386" xr:uid="{02C077D4-084C-49EC-8CEB-253639E24F6A}"/>
+    <cellStyle name="Moneda 34" xfId="387" xr:uid="{6F94E589-EA00-47EF-8C6F-6455C52FE025}"/>
+    <cellStyle name="Moneda 35" xfId="388" xr:uid="{448A6315-A6B1-4DDE-B313-36BB98AACF97}"/>
+    <cellStyle name="Moneda 36" xfId="389" xr:uid="{F760C08B-DBA4-4EFA-8E81-C23B84654DB4}"/>
+    <cellStyle name="Moneda 37" xfId="390" xr:uid="{1BC37208-310F-4810-B03C-A940F5F89634}"/>
+    <cellStyle name="Moneda 38" xfId="391" xr:uid="{53E9063C-6241-436C-84B0-C7F0F229DF95}"/>
+    <cellStyle name="Moneda 39" xfId="392" xr:uid="{B4E1011B-6815-4692-B4E4-3967336FDCD9}"/>
+    <cellStyle name="Moneda 4" xfId="125" xr:uid="{0B5D4054-118F-4828-AE5B-6B959D4DEC9F}"/>
+    <cellStyle name="Moneda 40" xfId="393" xr:uid="{62C38A50-60BF-4F27-A3A8-60CA4E281CF2}"/>
+    <cellStyle name="Moneda 41" xfId="394" xr:uid="{B8FAFA9B-34DE-4015-8C56-EE840FDAFB15}"/>
+    <cellStyle name="Moneda 42" xfId="395" xr:uid="{589C0364-9E6E-47D7-A91E-63098E1D60E0}"/>
+    <cellStyle name="Moneda 43" xfId="396" xr:uid="{7E8C3F0C-B667-45FF-B3C3-A2EA551932D0}"/>
+    <cellStyle name="Moneda 44" xfId="397" xr:uid="{7A698FBB-CDD9-4D4E-8FF9-03D759A0B123}"/>
+    <cellStyle name="Moneda 45" xfId="398" xr:uid="{6EE34F7D-36EF-4908-9D68-6068368B542F}"/>
+    <cellStyle name="Moneda 46" xfId="399" xr:uid="{917DC39F-FB0C-4CC2-9DC7-CEFE55BA46DD}"/>
+    <cellStyle name="Moneda 47" xfId="400" xr:uid="{A2DFDA78-F628-43EE-8825-BCDE868E551A}"/>
+    <cellStyle name="Moneda 48" xfId="401" xr:uid="{45C0F9E9-362B-496C-A8FE-F223EEF6243E}"/>
+    <cellStyle name="Moneda 49" xfId="402" xr:uid="{373513D7-61EC-44EC-A129-EFB0D098F7C4}"/>
+    <cellStyle name="Moneda 5" xfId="126" xr:uid="{B4D96E83-C374-459D-8EB7-3319C4744A18}"/>
+    <cellStyle name="Moneda 50" xfId="403" xr:uid="{5EA935CF-2D8A-4739-AC29-A37CACE37556}"/>
+    <cellStyle name="Moneda 51" xfId="404" xr:uid="{5DBD10C0-3FC1-4FCD-8426-85D35D05B3E0}"/>
+    <cellStyle name="Moneda 52" xfId="405" xr:uid="{B22FA8FA-4592-4696-A91A-31738FECC2C9}"/>
+    <cellStyle name="Moneda 53" xfId="406" xr:uid="{59E2214F-52BD-4FB5-B6F8-33A7DAEF742D}"/>
+    <cellStyle name="Moneda 54" xfId="407" xr:uid="{766E4FB7-6F08-4BD5-A477-CA2191B0FA0A}"/>
+    <cellStyle name="Moneda 55" xfId="408" xr:uid="{C8F9D6B9-3D88-448D-B59C-A2AA5FB76215}"/>
+    <cellStyle name="Moneda 56" xfId="409" xr:uid="{5CDF3B8E-3901-4102-9DA3-770E63016189}"/>
+    <cellStyle name="Moneda 57" xfId="410" xr:uid="{82255A7C-B09E-451E-9C26-527DE045E21E}"/>
+    <cellStyle name="Moneda 58" xfId="411" xr:uid="{002DBC62-371B-43C3-905F-08C216CA0062}"/>
+    <cellStyle name="Moneda 59" xfId="412" xr:uid="{CBA724A5-DC45-4971-B204-DF6FA005B62A}"/>
+    <cellStyle name="Moneda 6" xfId="127" xr:uid="{4A4D3B87-1884-46CD-8265-3CA211BAB006}"/>
+    <cellStyle name="Moneda 60" xfId="413" xr:uid="{92897976-A7DD-4C89-8E9E-043F2F14FE84}"/>
+    <cellStyle name="Moneda 61" xfId="414" xr:uid="{E458FF83-6862-4793-9F7E-AB892CD54988}"/>
+    <cellStyle name="Moneda 62" xfId="415" xr:uid="{39211068-0F2F-4651-BEB0-8A37586C4757}"/>
+    <cellStyle name="Moneda 63" xfId="416" xr:uid="{CB6368BD-7A1A-428F-8949-8A76EEB90EEF}"/>
+    <cellStyle name="Moneda 64" xfId="417" xr:uid="{7C7D5C07-7C0D-44C3-B4CB-A692D16D81A1}"/>
+    <cellStyle name="Moneda 65" xfId="418" xr:uid="{E70D9008-4AD7-4375-8FB1-F93FC54BD6CC}"/>
+    <cellStyle name="Moneda 66" xfId="419" xr:uid="{55B86003-2672-46A3-A35E-CD4A17B58E9F}"/>
+    <cellStyle name="Moneda 67" xfId="420" xr:uid="{90107E38-A1A6-4FC1-AA79-92554C8D2C79}"/>
+    <cellStyle name="Moneda 68" xfId="421" xr:uid="{44907EE7-EECC-4372-A5D2-CC92EDE3B8C6}"/>
+    <cellStyle name="Moneda 69" xfId="422" xr:uid="{8C723A2D-B140-4D7B-8A80-4AAACF2493E2}"/>
+    <cellStyle name="Moneda 7" xfId="128" xr:uid="{9EF76613-2CEC-432B-BB1D-E39B06B53225}"/>
+    <cellStyle name="Moneda 70" xfId="423" xr:uid="{0D14D905-6047-4183-82C3-70B98CDF3C28}"/>
+    <cellStyle name="Moneda 71" xfId="424" xr:uid="{2A4F3EE1-24B0-4724-B2FE-C417CE1B2211}"/>
+    <cellStyle name="Moneda 72" xfId="425" xr:uid="{92DE947C-4083-4256-BD3B-0B936A57E034}"/>
+    <cellStyle name="Moneda 73" xfId="426" xr:uid="{54C73DC9-1B9B-499A-9592-2632E5277581}"/>
+    <cellStyle name="Moneda 74" xfId="427" xr:uid="{AF75E995-7A2C-4CA5-B3CA-ED7D66F1B634}"/>
+    <cellStyle name="Moneda 75" xfId="428" xr:uid="{1D898573-EE59-48F0-8496-8591382F8892}"/>
+    <cellStyle name="Moneda 8" xfId="195" xr:uid="{C0B90446-D81E-4024-B6F4-BF1D94D72FD6}"/>
+    <cellStyle name="Moneda 9" xfId="196" xr:uid="{708339EB-DB61-4335-BA8E-BDDB521E6540}"/>
+    <cellStyle name="Neutral 2" xfId="38" xr:uid="{2D2D1C60-0974-4129-9129-01DC5451A196}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 10" xfId="72" xr:uid="{4EAF1BC2-7121-44F1-B4F7-C5CFDA11B12C}"/>
+    <cellStyle name="Normal 11" xfId="74" xr:uid="{AB215E47-95C1-47B0-B941-401FFE9BB871}"/>
+    <cellStyle name="Normal 12" xfId="76" xr:uid="{F45A2D29-0F6C-4E0D-B146-E0D110E0EF09}"/>
+    <cellStyle name="Normal 12 2" xfId="80" xr:uid="{B05B218F-6302-4943-9CFF-77E12DD53F82}"/>
+    <cellStyle name="Normal 13" xfId="78" xr:uid="{D950317A-395D-477E-8005-4956AEA06A8E}"/>
+    <cellStyle name="Normal 14" xfId="97" xr:uid="{B19A7CF7-B2CC-458B-9AC0-5FC2B69FEB1A}"/>
+    <cellStyle name="Normal 15" xfId="99" xr:uid="{D89F4A66-8A9B-4EF8-8559-E7C2D99DB93E}"/>
+    <cellStyle name="Normal 16" xfId="101" xr:uid="{5D938E42-442A-4362-AF90-4EA0D24D8D81}"/>
+    <cellStyle name="Normal 17" xfId="103" xr:uid="{2BCE6908-5F6F-4B42-91AF-E6022C01E51F}"/>
+    <cellStyle name="Normal 18" xfId="105" xr:uid="{69367441-3446-41B9-A464-2FA770E7E9C2}"/>
+    <cellStyle name="Normal 19" xfId="107" xr:uid="{DD375DA0-8D5B-42C1-9DFD-228707876D7B}"/>
+    <cellStyle name="Normal 2" xfId="48" xr:uid="{1721DC64-2D5F-4D6E-930B-51707720949C}"/>
+    <cellStyle name="Normal 2 10" xfId="140" xr:uid="{58CA1B87-3EC3-401C-B7E5-030A2D40F3A5}"/>
+    <cellStyle name="Normal 2 11" xfId="221" xr:uid="{B428867D-8730-4228-B090-4AFCA4A687D1}"/>
+    <cellStyle name="Normal 2 2" xfId="69" xr:uid="{2A86A124-402E-4862-A411-99AF394C92DA}"/>
+    <cellStyle name="Normal 2 2 2" xfId="136" xr:uid="{CB122AA5-131B-4BCD-9021-98407FAE8D41}"/>
+    <cellStyle name="Normal 2 2 3" xfId="222" xr:uid="{F884DC22-A070-4ED7-97EA-E8F100EBF687}"/>
+    <cellStyle name="Normal 2 3" xfId="66" xr:uid="{456CEC39-B249-43D0-8B88-C1FF534F396E}"/>
+    <cellStyle name="Normal 2 3 2" xfId="137" xr:uid="{ECDF389E-44EE-49A1-AD31-884BC7340B09}"/>
+    <cellStyle name="Normal 2 4" xfId="139" xr:uid="{2BC37486-BF6E-4196-BA5E-F6C50D4C03DD}"/>
+    <cellStyle name="Normal 2 5" xfId="165" xr:uid="{FA22BCF7-57A4-46BF-9CEB-ED9A3AFC65C4}"/>
+    <cellStyle name="Normal 2 6" xfId="171" xr:uid="{E7D52698-F916-4E23-AEBD-1444CD5352FF}"/>
+    <cellStyle name="Normal 2 7" xfId="176" xr:uid="{6D76A348-045D-4533-8431-CF5937276194}"/>
+    <cellStyle name="Normal 2 8" xfId="182" xr:uid="{9B7FA36C-48CF-4E8F-8733-DE3883B0E53A}"/>
+    <cellStyle name="Normal 2 9" xfId="186" xr:uid="{062A4D30-FC80-4592-B8B1-75E70CAAE81E}"/>
+    <cellStyle name="Normal 20" xfId="109" xr:uid="{C5D4E733-5DAC-4763-ABD3-EBBDF64398D8}"/>
+    <cellStyle name="Normal 21" xfId="111" xr:uid="{BCFE3018-2D14-42C7-A56E-AEA1FF308EF3}"/>
+    <cellStyle name="Normal 22" xfId="113" xr:uid="{F0D78D77-2C53-4C72-8C63-0F80FB356F07}"/>
+    <cellStyle name="Normal 23" xfId="115" xr:uid="{44847DCC-967B-46D3-9BF9-4DD14BEA7840}"/>
+    <cellStyle name="Normal 24" xfId="117" xr:uid="{FAE756FB-E4F8-4B94-9B9B-F23963770FEE}"/>
+    <cellStyle name="Normal 25" xfId="119" xr:uid="{9A285CC4-AB1C-403E-8427-5560C858F602}"/>
+    <cellStyle name="Normal 26" xfId="121" xr:uid="{4D2DF8A9-205C-4F23-8234-2B156B98B6AB}"/>
+    <cellStyle name="Normal 27" xfId="123" xr:uid="{4A211BD3-8657-4857-BC16-D51622CC5861}"/>
+    <cellStyle name="Normal 28" xfId="45" xr:uid="{8AF2CF2B-F35C-4961-B1AA-495F623765D3}"/>
+    <cellStyle name="Normal 28 2" xfId="292" xr:uid="{3F2D6C85-76C8-44DD-8899-DBF6306301B8}"/>
+    <cellStyle name="Normal 29" xfId="294" xr:uid="{2EAB64D2-4A54-493B-9110-0F9ED2544347}"/>
+    <cellStyle name="Normal 3" xfId="50" xr:uid="{6E9EF77C-C001-46FC-A232-A69D5AF10D0A}"/>
+    <cellStyle name="Normal 3 2" xfId="68" xr:uid="{CBD90EC6-8FAC-4DEA-A319-41CFC7ABB013}"/>
+    <cellStyle name="Normal 3 2 2" xfId="163" xr:uid="{BFEAEC13-CA14-4359-AD5F-E6EF7857DB65}"/>
+    <cellStyle name="Normal 3 3" xfId="213" xr:uid="{672FAA7D-BBBC-4CAB-A3E4-24DDC2FB2468}"/>
+    <cellStyle name="Normal 30" xfId="296" xr:uid="{A3A8BA46-0498-4B76-88B8-8B1A85F39206}"/>
+    <cellStyle name="Normal 31" xfId="313" xr:uid="{7B2AC8A0-A095-4CDF-9580-F2E499F8C344}"/>
+    <cellStyle name="Normal 32" xfId="315" xr:uid="{9936E8F6-C278-4C8D-8020-5C4EC63B714F}"/>
+    <cellStyle name="Normal 33" xfId="317" xr:uid="{ADF8494E-D728-45C5-B1F9-1223E73AEA3A}"/>
+    <cellStyle name="Normal 34" xfId="319" xr:uid="{23F20361-DCB1-4A7A-8AC2-26C936C48D16}"/>
+    <cellStyle name="Normal 35" xfId="257" xr:uid="{4F706F13-C92A-443C-8433-D884636DC5C6}"/>
+    <cellStyle name="Normal 4" xfId="52" xr:uid="{9787108B-ACDB-4459-A3A2-9A6F71034951}"/>
+    <cellStyle name="Normal 4 2" xfId="138" xr:uid="{B6303C98-BD1F-4073-B900-69C8D7C4BCFD}"/>
+    <cellStyle name="Normal 4 2 2" xfId="376" xr:uid="{1EA056AC-7F5A-4837-822F-4EDC91133F3E}"/>
+    <cellStyle name="Normal 4 3" xfId="167" xr:uid="{90E4D0DD-2573-434A-85B5-B05C1C6B483F}"/>
+    <cellStyle name="Normal 4 4" xfId="178" xr:uid="{20925D0D-463F-4B48-AF63-1EC8C01570A2}"/>
+    <cellStyle name="Normal 4 5" xfId="250" xr:uid="{FE431AB4-1132-46AD-A1CE-6CD5B6FF8A96}"/>
+    <cellStyle name="Normal 5" xfId="54" xr:uid="{E35CA0E1-3D2A-4C45-B714-DA39AB40098A}"/>
+    <cellStyle name="Normal 5 2" xfId="134" xr:uid="{C4E92EFF-A329-4EA5-A38A-F15BA5B99827}"/>
+    <cellStyle name="Normal 6" xfId="56" xr:uid="{25F91E06-36F6-4686-99F0-B006133FD552}"/>
+    <cellStyle name="Normal 6 2" xfId="129" xr:uid="{15E4E730-9EEB-4986-8E76-FFA7534448FD}"/>
+    <cellStyle name="Normal 6 3" xfId="263" xr:uid="{2C218801-042F-47B2-9505-98865858B62C}"/>
+    <cellStyle name="Normal 7" xfId="58" xr:uid="{4FD422D4-57EA-4FAD-AEB4-9976BF535ACB}"/>
+    <cellStyle name="Normal 8" xfId="60" xr:uid="{E1FB1B28-3E72-459A-B265-6FBBD9B9406E}"/>
+    <cellStyle name="Normal 9" xfId="62" xr:uid="{6367556B-C500-4C9F-BA4C-D817F2ECD15E}"/>
+    <cellStyle name="Notas 2" xfId="67" xr:uid="{9BD6A2BE-1E8F-4142-BB35-3EC627A875EB}"/>
+    <cellStyle name="Notas 3" xfId="84" xr:uid="{F315B608-7423-4AA7-ACEF-BEB3E8838735}"/>
+    <cellStyle name="Notas 4" xfId="300" xr:uid="{D00C0308-BF55-4DDA-BCDC-46F5A01BFA7C}"/>
+    <cellStyle name="Porcentaje 2" xfId="47" xr:uid="{C7D0C856-C81B-4502-8112-46CDF7E6F0C1}"/>
+    <cellStyle name="Porcentaje 2 2" xfId="132" xr:uid="{DCD8A671-92F9-4955-A8F2-380CBCF091C9}"/>
+    <cellStyle name="Porcentaje 2 3" xfId="224" xr:uid="{225397E5-D6D9-4187-BD8B-6942995A507E}"/>
+    <cellStyle name="Porcentaje 2 4" xfId="223" xr:uid="{DECBD0DA-4AB8-473B-9186-0D7E216A02A2}"/>
+    <cellStyle name="Porcentaje 3" xfId="225" xr:uid="{74D78EDA-7C5A-4416-ABAB-BC3BC5247256}"/>
+    <cellStyle name="Porcentaje 4" xfId="258" xr:uid="{E1BB59E0-0F80-45E8-A458-430DCB8BFD19}"/>
+    <cellStyle name="Porcentaje 4 2" xfId="377" xr:uid="{BC9A9168-0195-4D60-BBC1-FA4CE4DEAEFC}"/>
+    <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Texto explicativo" xfId="15" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Título" xfId="2" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Título 2" xfId="4" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Título 3" xfId="5" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="16" builtinId="25" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -214,6 +1522,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -533,7 +1845,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5743232F-8CE5-4C8B-B889-62F0D37F13AD}">
-  <dimension ref="A1:Q312"/>
+  <dimension ref="A1:Q318"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="1"/>
@@ -16983,19 +18295,19 @@
         <v>46174</v>
       </c>
       <c r="B311">
-        <v>21</v>
-      </c>
-      <c r="C311">
-        <v>103175000</v>
+        <v>19</v>
+      </c>
+      <c r="C311" s="16">
+        <v>94675000</v>
       </c>
       <c r="D311">
-        <v>9</v>
-      </c>
-      <c r="E311">
-        <v>73040</v>
+        <v>7</v>
+      </c>
+      <c r="E311" s="16">
+        <v>56816</v>
       </c>
       <c r="F311" s="9">
-        <v>0.42857142857142855</v>
+        <v>0.37</v>
       </c>
       <c r="G311">
         <v>27</v>
@@ -17007,7 +18319,7 @@
         <v>4</v>
       </c>
       <c r="J311">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K311">
         <v>0</v>
@@ -17033,22 +18345,22 @@
     </row>
     <row r="312" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A312" s="1">
-        <v>46147</v>
+        <v>46175</v>
       </c>
       <c r="B312">
-        <v>28</v>
-      </c>
-      <c r="C312">
-        <v>80760000</v>
+        <v>27</v>
+      </c>
+      <c r="C312" s="16">
+        <v>75260000</v>
       </c>
       <c r="D312">
-        <v>14</v>
-      </c>
-      <c r="E312">
-        <v>113682</v>
+        <v>12</v>
+      </c>
+      <c r="E312" s="16">
+        <v>97442</v>
       </c>
       <c r="F312" s="9">
-        <v>0.5</v>
+        <v>0.44</v>
       </c>
       <c r="G312">
         <v>99</v>
@@ -17057,10 +18369,10 @@
         <v>378699606</v>
       </c>
       <c r="I312">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J312">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K312">
         <v>0</v>
@@ -17069,7 +18381,7 @@
         <v>0</v>
       </c>
       <c r="M312">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N312">
         <v>51</v>
@@ -17081,6 +18393,324 @@
         <v>0</v>
       </c>
       <c r="Q312">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="313" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A313" s="1">
+        <v>46176</v>
+      </c>
+      <c r="B313">
+        <v>35</v>
+      </c>
+      <c r="C313" s="16">
+        <v>211425500</v>
+      </c>
+      <c r="D313">
+        <v>14</v>
+      </c>
+      <c r="E313" s="16">
+        <v>113832</v>
+      </c>
+      <c r="F313" s="9">
+        <v>0.4</v>
+      </c>
+      <c r="G313">
+        <v>101</v>
+      </c>
+      <c r="H313" s="11">
+        <v>395205507</v>
+      </c>
+      <c r="I313">
+        <v>2</v>
+      </c>
+      <c r="J313">
+        <v>0</v>
+      </c>
+      <c r="K313">
+        <v>0</v>
+      </c>
+      <c r="L313">
+        <v>0</v>
+      </c>
+      <c r="M313">
+        <v>1</v>
+      </c>
+      <c r="N313">
+        <v>40</v>
+      </c>
+      <c r="O313">
+        <v>44</v>
+      </c>
+      <c r="P313">
+        <v>0</v>
+      </c>
+      <c r="Q313">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="314" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A314" s="1">
+        <v>46177</v>
+      </c>
+      <c r="B314">
+        <v>53</v>
+      </c>
+      <c r="C314" s="16">
+        <v>262100000</v>
+      </c>
+      <c r="D314">
+        <v>23</v>
+      </c>
+      <c r="E314" s="16">
+        <v>187142</v>
+      </c>
+      <c r="F314" s="9">
+        <v>0.43</v>
+      </c>
+      <c r="G314">
+        <v>98</v>
+      </c>
+      <c r="H314" s="11">
+        <v>314847525</v>
+      </c>
+      <c r="I314">
+        <v>3</v>
+      </c>
+      <c r="J314">
+        <v>2</v>
+      </c>
+      <c r="K314">
+        <v>0</v>
+      </c>
+      <c r="L314">
+        <v>0</v>
+      </c>
+      <c r="M314">
+        <v>5</v>
+      </c>
+      <c r="N314">
+        <v>61</v>
+      </c>
+      <c r="O314">
+        <v>31</v>
+      </c>
+      <c r="P314">
+        <v>0</v>
+      </c>
+      <c r="Q314">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="315" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A315" s="1">
+        <v>46178</v>
+      </c>
+      <c r="B315">
+        <v>35</v>
+      </c>
+      <c r="C315" s="16">
+        <v>159790000</v>
+      </c>
+      <c r="D315">
+        <v>11</v>
+      </c>
+      <c r="E315" s="16">
+        <v>89536</v>
+      </c>
+      <c r="F315" s="9">
+        <v>0.31</v>
+      </c>
+      <c r="G315">
+        <v>70</v>
+      </c>
+      <c r="H315" s="11">
+        <v>181815190</v>
+      </c>
+      <c r="I315">
+        <v>5</v>
+      </c>
+      <c r="J315">
+        <v>1</v>
+      </c>
+      <c r="K315">
+        <v>0</v>
+      </c>
+      <c r="L315">
+        <v>0</v>
+      </c>
+      <c r="M315">
+        <v>2</v>
+      </c>
+      <c r="N315">
+        <v>35</v>
+      </c>
+      <c r="O315">
+        <v>40</v>
+      </c>
+      <c r="P315">
+        <v>0</v>
+      </c>
+      <c r="Q315">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="316" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A316" s="1">
+        <v>46181</v>
+      </c>
+      <c r="B316">
+        <v>27</v>
+      </c>
+      <c r="C316" s="16">
+        <v>177035000</v>
+      </c>
+      <c r="D316">
+        <v>13</v>
+      </c>
+      <c r="E316" s="16">
+        <v>105927</v>
+      </c>
+      <c r="F316" s="9">
+        <v>0.48</v>
+      </c>
+      <c r="G316">
+        <v>77</v>
+      </c>
+      <c r="H316" s="11">
+        <v>259868252</v>
+      </c>
+      <c r="I316">
+        <v>5</v>
+      </c>
+      <c r="J316">
+        <v>0</v>
+      </c>
+      <c r="K316">
+        <v>0</v>
+      </c>
+      <c r="L316">
+        <v>0</v>
+      </c>
+      <c r="M316">
+        <v>0</v>
+      </c>
+      <c r="N316">
+        <v>31</v>
+      </c>
+      <c r="O316">
+        <v>37</v>
+      </c>
+      <c r="P316">
+        <v>0</v>
+      </c>
+      <c r="Q316">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="317" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A317" s="1">
+        <v>46182</v>
+      </c>
+      <c r="B317">
+        <v>26</v>
+      </c>
+      <c r="C317">
+        <v>159570000</v>
+      </c>
+      <c r="D317">
+        <v>12</v>
+      </c>
+      <c r="E317">
+        <v>97836</v>
+      </c>
+      <c r="F317" s="9">
+        <v>0.46</v>
+      </c>
+      <c r="G317">
+        <v>72</v>
+      </c>
+      <c r="H317" s="11">
+        <v>273532717</v>
+      </c>
+      <c r="I317">
+        <v>3</v>
+      </c>
+      <c r="J317">
+        <v>1</v>
+      </c>
+      <c r="K317">
+        <v>0</v>
+      </c>
+      <c r="L317">
+        <v>0</v>
+      </c>
+      <c r="M317">
+        <v>6</v>
+      </c>
+      <c r="N317">
+        <v>41</v>
+      </c>
+      <c r="O317">
+        <v>19</v>
+      </c>
+      <c r="P317">
+        <v>0</v>
+      </c>
+      <c r="Q317">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="318" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A318" s="1">
+        <v>46183</v>
+      </c>
+      <c r="B318">
+        <v>36</v>
+      </c>
+      <c r="C318">
+        <v>122122000</v>
+      </c>
+      <c r="D318">
+        <v>19</v>
+      </c>
+      <c r="E318">
+        <v>154909</v>
+      </c>
+      <c r="F318" s="9">
+        <v>0.53</v>
+      </c>
+      <c r="G318">
+        <v>101</v>
+      </c>
+      <c r="H318" s="11">
+        <v>457400070</v>
+      </c>
+      <c r="I318">
+        <v>3</v>
+      </c>
+      <c r="J318">
+        <v>0</v>
+      </c>
+      <c r="K318">
+        <v>0</v>
+      </c>
+      <c r="L318">
+        <v>0</v>
+      </c>
+      <c r="M318">
+        <v>12</v>
+      </c>
+      <c r="N318">
+        <v>19</v>
+      </c>
+      <c r="O318">
+        <v>38</v>
+      </c>
+      <c r="P318">
+        <v>0</v>
+      </c>
+      <c r="Q318">
         <v>0</v>
       </c>
     </row>

</xml_diff>